<commit_message>
Minor changes with some map changes
</commit_message>
<xml_diff>
--- a/data/lab/combined.results.xlsx
+++ b/data/lab/combined.results.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/profbabykangaroo/Library/Mobile Documents/com~apple~CloudDocs/Core/Server Files/swordfern/data/lab/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/professorbabykangaroo/Library/Mobile Documents/com~apple~CloudDocs/Core/Server Files/swordfern/data/lab/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0F876CE-2BFB-4B45-83F1-0C1CBF93AC65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA07F533-EDDD-9E41-878E-45DE992AA978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{10D213AB-7268-DA4E-BB0F-4ADD01F7F431}"/>
   </bookViews>
   <sheets>
     <sheet name="combined.results.copy" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'combined.results.copy'!$A$1:$BA$248</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -3589,6 +3592,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DA4AB90-CDE7-6849-A0DD-CF391E774401}">
   <dimension ref="A1:BA248"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="23.83203125" customWidth="1"/>
+    <col min="11" max="11" width="30.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:53" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
@@ -13063,13 +13070,13 @@
         <v>105</v>
       </c>
       <c r="AA70" t="s">
-        <v>105</v>
+        <v>367</v>
       </c>
       <c r="AB70" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="AC70" t="s">
-        <v>105</v>
+        <v>27</v>
       </c>
       <c r="AD70" t="s">
         <v>368</v>
@@ -13378,13 +13385,13 @@
         <v>105</v>
       </c>
       <c r="AA73" t="s">
-        <v>105</v>
+        <v>367</v>
       </c>
       <c r="AB73" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="AC73" t="s">
-        <v>105</v>
+        <v>27</v>
       </c>
       <c r="AD73" t="s">
         <v>374</v>
@@ -36907,6 +36914,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:BA248" xr:uid="{7DA4AB90-CDE7-6849-A0DD-CF391E774401}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>